<commit_message>
Fix bulk upload processing and checkout validation
</commit_message>
<xml_diff>
--- a/templates/compliantuk-portfolio-template.xlsx
+++ b/templates/compliantuk-portfolio-template.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Upload" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CompliantUK Bulk Upload" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,28 +27,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001d4ed8"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -57,24 +40,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001d4ed8"/>
-        <bgColor rgb="001d4ed8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00f8fafc"/>
-        <bgColor rgb="00f8fafc"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00ffffff"/>
-        <bgColor rgb="00ffffff"/>
+        <fgColor rgb="001D4ED8"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -82,38 +52,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00e2e8f0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00e2e8f0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00e2e8f0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00e2e8f0"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -479,28 +426,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="28" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>landlord_first</t>
@@ -581,110 +534,187 @@
           <t>tenant4_email</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>tenant5_first</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>tenant5_last</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>tenant5_email</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>tenant6_first</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>tenant6_last</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>tenant6_email</t>
+        </is>
+      </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>John</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Smith</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>john.smith@email.com</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>12 Oak Street, London, E1 2AB</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Alice</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Johnson</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>alice@email.com</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>alice@example.com</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>Bob</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Williams</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>bob@email.com</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>bob@example.com</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Carla</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Reed</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>carla@example.com</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Singh</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>david@example.com</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Ella</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Patel</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>ella@example.com</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Sarah</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Brown</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>sarah.brown@gmail.com</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>sarah.brown@example.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>45 Maple Avenue, Manchester, M1 3CD</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Tom</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Davis</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>tom.davis@email.com</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr"/>
-      <c r="L3" s="3" t="inlineStr"/>
-      <c r="M3" s="3" t="inlineStr"/>
-      <c r="N3" s="3" t="inlineStr"/>
-      <c r="O3" s="3" t="inlineStr"/>
-      <c r="P3" s="3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>tom.davis@example.com</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -697,79 +727,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>CompliantUK Portfolio Upload Template</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>CompliantUK portfolio upload instructions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Use one row per property. Tenant 1 is required; tenants 2-6 are optional. Invalid tenant emails will be skipped and reported before payment.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>INSTRUCTIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>1. Fill in one row per tenancy (one property).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>2. landlord_first, landlord_last, landlord_email, property_address are REQUIRED for every row.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>3. At least tenant1_first, tenant1_last, tenant1_email are REQUIRED.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>4. Tenants 2, 3 and 4 are optional — leave blank if not applicable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>5. Maximum 4 tenants per property row.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>6. Do not change the column headers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>7. Save as .xlsx or .csv before uploading.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>8. Delete the example rows before uploading.</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Columns must keep the exact header names in row 1.</t>
         </is>
       </c>
     </row>

</xml_diff>